<commit_message>
changing the interfaces organisation
</commit_message>
<xml_diff>
--- a/saves/bulletins.xlsx
+++ b/saves/bulletins.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Registre bulletins" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registre bulletins'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registre bulletins'!$A$1:$L$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -861,200 +861,8 @@
         <v>3005.62</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>ABIDI</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>MED aziz</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>developpeur</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>N005</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>2900</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>359.67</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>1017.13</v>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>2541.19</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>HWAWI</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>HADIL</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>responsable logistique</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>N006</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>3800</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>480</v>
-      </c>
-      <c r="J9" s="8" t="n">
-        <v>393.45</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>1145.93</v>
-      </c>
-      <c r="L9" s="9" t="n">
-        <v>2746.61</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>ABIDI</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>MED aziz</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>developpeur</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>N007</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>2900</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>359.67</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>1017.13</v>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>2541.19</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BRAHMI </t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>HAMZA</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chef projet </t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>N008</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H11" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>380</v>
-      </c>
-      <c r="J11" s="8" t="n">
-        <v>586.1</v>
-      </c>
-      <c r="K11" s="8" t="n">
-        <v>1880.41</v>
-      </c>
-      <c r="L11" s="9" t="n">
-        <v>3917.99</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L11"/>
+  <autoFilter ref="A1:L7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixing the comparison button
</commit_message>
<xml_diff>
--- a/saves/bulletins.xlsx
+++ b/saves/bulletins.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Registre bulletins" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registre bulletins'!$A$1:$L$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registre bulletins'!$A$1:$M$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,13 +494,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -509,6 +509,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="29" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -572,6 +573,11 @@
           <t>Salaire Net</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Date Ajout</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -594,7 +600,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>N001</t>
+          <t>N002</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -606,19 +612,24 @@
         <v>2900</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>480</v>
+        <v>1000</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>310.97</v>
+        <v>359.67</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>831.46</v>
+        <v>1017.13</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>2245.07</v>
+        <v>2541.19</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>15 Aout 2026 - 12:39</t>
+        </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -642,7 +653,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>N006</t>
+          <t>N003</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -651,218 +662,31 @@
         </is>
       </c>
       <c r="G3" s="6" t="n">
-        <v>2900</v>
+        <v>2300</v>
       </c>
       <c r="H3" s="6" t="n">
         <v>12</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>1000</v>
+        <v>450</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>359.67</v>
+        <v>254.1</v>
       </c>
       <c r="K3" s="8" t="n">
-        <v>1017.13</v>
+        <v>614.63</v>
       </c>
       <c r="L3" s="9" t="n">
-        <v>2541.19</v>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>BRAHMI</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>HAMZA</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CHEF PROJET </t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>N002</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H4" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="I4" s="2" t="n">
-        <v>1000</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>644.25</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>2102.13</v>
-      </c>
-      <c r="L4" s="5" t="n">
-        <v>4271.61</v>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>BRAHMI</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>HAMZA</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CHEF PROJET </t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>N007</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>2000</v>
-      </c>
-      <c r="J5" s="8" t="n">
-        <v>737.7</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>2458.43</v>
-      </c>
-      <c r="L5" s="9" t="n">
-        <v>4839.86</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KADRI </t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>NACER</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">chef projet </t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>N003</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>500</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>597.53</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>1923.98</v>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>3987.49</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BESBES </t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>MARIEM</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">RH </t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>N004</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Aout 2026</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>4500</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>250</v>
-      </c>
-      <c r="J7" s="8" t="n">
-        <v>436.05</v>
-      </c>
-      <c r="K7" s="8" t="n">
-        <v>1308.33</v>
-      </c>
-      <c r="L7" s="9" t="n">
-        <v>3005.62</v>
+        <v>1899.26</v>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
+          <t>15 october 2025 - 12:42</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L7"/>
+  <autoFilter ref="A1:M3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>